<commit_message>
All unit tests passing with new reg files
</commit_message>
<xml_diff>
--- a/src/test/java/simpaths/testinput/reg_eq5d.xlsx
+++ b/src/test/java/simpaths/testinput/reg_eq5d.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\andy_local\SimPaths project files\SimPaths\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\andy_local\SimPaths project files\SimPaths\src\test\java\simpaths\testinput\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7731E325-0622-4050-B24A-A7B4DDB31076}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FD4F519-819D-4B03-8F5D-5EE0DD950912}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{8A9A3AE8-34F1-4C3E-9682-3C69CFBA3626}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8A9A3AE8-34F1-4C3E-9682-3C69CFBA3626}"/>
   </bookViews>
   <sheets>
-    <sheet name="UK_EQ5D_lawrence" sheetId="1" r:id="rId1"/>
-    <sheet name="UK_EQ5D_franks" sheetId="2" r:id="rId2"/>
+    <sheet name="EQ5D_lawrence" sheetId="1" r:id="rId1"/>
+    <sheet name="EQ5D_franks" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>

<commit_message>
restore `src/test` and `pom.xml` to develop version
</commit_message>
<xml_diff>
--- a/src/test/java/simpaths/testinput/reg_eq5d.xlsx
+++ b/src/test/java/simpaths/testinput/reg_eq5d.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\andy_local\SimPaths project files\SimPaths\src\test\java\simpaths\testinput\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\andy_local\SimPaths project files\SimPaths\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FD4F519-819D-4B03-8F5D-5EE0DD950912}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7731E325-0622-4050-B24A-A7B4DDB31076}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8A9A3AE8-34F1-4C3E-9682-3C69CFBA3626}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{8A9A3AE8-34F1-4C3E-9682-3C69CFBA3626}"/>
   </bookViews>
   <sheets>
-    <sheet name="EQ5D_lawrence" sheetId="1" r:id="rId1"/>
-    <sheet name="EQ5D_franks" sheetId="2" r:id="rId2"/>
+    <sheet name="UK_EQ5D_lawrence" sheetId="1" r:id="rId1"/>
+    <sheet name="UK_EQ5D_franks" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>